<commit_message>
add update and remove invoice
</commit_message>
<xml_diff>
--- a/cache/sepidar_food_code.xlsx
+++ b/cache/sepidar_food_code.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24701"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dorsa-Co\Desktop\temp\pichNew\cache\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\milad\Desktop\SeketalaFolder\seketalaNew\cache\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76C493B9-6899-4B46-A5DB-C2CC65FE7ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{867BA7FC-8662-4D7A-8D54-85A5E72CFF21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4110" yWindow="3435" windowWidth="21540" windowHeight="11355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="633">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="635">
   <si>
     <t>كد</t>
   </si>
@@ -1924,6 +1924,12 @@
   </si>
   <si>
     <t>قوطي زيرو کوکا با ليوان</t>
+  </si>
+  <si>
+    <t>لیموناد ۲۵۰ سیسی لاکی</t>
+  </si>
+  <si>
+    <t xml:space="preserve">لیموناد قوطی خوشگوار </t>
   </si>
 </sst>
 </file>
@@ -5644,11 +5650,23 @@
       <c r="Z342" s="7"/>
       <c r="AB342" s="7"/>
     </row>
-    <row r="343" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A343">
+        <v>2800013</v>
+      </c>
+      <c r="B343" s="9" t="s">
+        <v>633</v>
+      </c>
       <c r="Z343" s="7"/>
       <c r="AB343" s="7"/>
     </row>
-    <row r="344" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A344">
+        <v>1100076</v>
+      </c>
+      <c r="B344" s="9" t="s">
+        <v>634</v>
+      </c>
       <c r="Z344" s="7"/>
       <c r="AB344" s="7"/>
     </row>

</xml_diff>